<commit_message>
feat: add floating point library, restructure tools
- program/floatingpoint: IEEE-754 binary32 soft-float header (add/sub/mul/div,
  str2f/f2str) with ISA-32 emulator and test runner
- tools: mirror src layout (assembler/linker/common/hexdump), add SYNTAX.md,
  BUGS.md, dlnk; update dasm/hexdump binaries
- cpu-32 test / flush-mux WIP, ISA.md, docs and todo updates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tqdin4SKwXxay7Y3C1dxMN
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1F13FD-A61F-46C4-95A6-76D75D0D5CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A77CC6D-249D-47F7-835D-0D6500569CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="1905" windowWidth="28800" windowHeight="12915" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="211">
   <si>
     <t>opcode</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -369,10 +369,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>flush</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>intervec</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -405,10 +401,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>inval</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>name</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -821,14 +813,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>8. mode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>7. none</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>6. none</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -853,19 +837,48 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>mode means select all content</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>id(EXT)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>flush cache[base+m]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>invalidate cache[base+m]</t>
+    <t>all: all in cache, md: flush/inval</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7. all</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8. md</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flush/inval cache[base+m]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>atom</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>len</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u.u</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>atomize following</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>register
+EXT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>extra</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -914,7 +927,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -938,11 +951,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -951,9 +966,13 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -962,11 +981,13 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -981,7 +1002,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -993,10 +1014,10 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -1008,28 +1029,13 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1044,54 +1050,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -1129,10 +1087,47 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -1145,7 +1140,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
@@ -1156,30 +1151,17 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
@@ -1190,7 +1172,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
@@ -1199,48 +1181,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -1252,7 +1197,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1277,31 +1222,100 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1313,85 +1327,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1740,78 +1676,78 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="38"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="39"/>
+      <c r="B6" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="22"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="40"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="42"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="25"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="43"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="44"/>
-      <c r="J8" s="44"/>
-      <c r="K8" s="44"/>
-      <c r="L8" s="44"/>
-      <c r="M8" s="44"/>
-      <c r="N8" s="44"/>
-      <c r="O8" s="45"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
+      <c r="O8" s="28"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="36"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="18"/>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>46</v>
@@ -1831,11 +1767,11 @@
       <c r="H10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="I10" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
       <c r="L10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1843,17 +1779,17 @@
         <v>39</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1869,15 +1805,15 @@
         <v>12</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I11" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I11" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16" t="s">
-        <v>105</v>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17" t="s">
+        <v>103</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>26</v>
@@ -1887,14 +1823,14 @@
         <v>gen[0]</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C12" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C12" s="17"/>
       <c r="D12" s="3" t="str">
         <f t="shared" ref="D12:D36" si="1">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D11)+1))</f>
         <v>01</v>
@@ -1909,14 +1845,14 @@
         <v>12</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I12" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I12" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
       <c r="M12" s="3" t="str">
         <f t="shared" ref="M12:M42" si="2">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M11)+1))</f>
         <v>01</v>
@@ -1925,15 +1861,15 @@
         <f t="shared" si="0"/>
         <v>gen[1]</v>
       </c>
-      <c r="O12" s="36" t="s">
-        <v>153</v>
+      <c r="O12" s="18" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C13" s="17"/>
       <c r="D13" s="3" t="str">
         <f t="shared" si="1"/>
         <v>02</v>
@@ -1944,16 +1880,16 @@
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16" t="s">
+      <c r="H13" s="17"/>
+      <c r="I13" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="J13" s="16"/>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
       <c r="M13" s="3" t="str">
         <f t="shared" si="2"/>
         <v>02</v>
@@ -1962,13 +1898,13 @@
         <f t="shared" si="0"/>
         <v>gen[2]</v>
       </c>
-      <c r="O13" s="36"/>
+      <c r="O13" s="18"/>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C14" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C14" s="17"/>
       <c r="D14" s="3" t="str">
         <f t="shared" si="1"/>
         <v>03</v>
@@ -1983,14 +1919,14 @@
         <v>12</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I14" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I14" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
       <c r="M14" s="3" t="str">
         <f t="shared" si="2"/>
         <v>03</v>
@@ -1999,13 +1935,13 @@
         <f t="shared" si="0"/>
         <v>gen[3]</v>
       </c>
-      <c r="O14" s="36"/>
+      <c r="O14" s="18"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C15" s="17"/>
       <c r="D15" s="3" t="str">
         <f t="shared" si="1"/>
         <v>04</v>
@@ -2020,14 +1956,14 @@
         <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I15" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
       <c r="M15" s="3" t="str">
         <f t="shared" si="2"/>
         <v>04</v>
@@ -2036,25 +1972,25 @@
         <f t="shared" si="0"/>
         <v>gen[4]</v>
       </c>
-      <c r="O15" s="36"/>
-      <c r="U15" s="28"/>
-      <c r="V15" s="28"/>
-      <c r="W15" s="28"/>
-      <c r="X15" s="28"/>
-      <c r="Y15" s="28"/>
-      <c r="Z15" s="28"/>
-      <c r="AA15" s="28"/>
-      <c r="AB15" s="28"/>
-      <c r="AC15" s="28"/>
-      <c r="AD15" s="28"/>
-      <c r="AF15" s="28"/>
-      <c r="AG15" s="28"/>
+      <c r="O15" s="18"/>
+      <c r="U15" s="16"/>
+      <c r="V15" s="16"/>
+      <c r="W15" s="16"/>
+      <c r="X15" s="16"/>
+      <c r="Y15" s="16"/>
+      <c r="Z15" s="16"/>
+      <c r="AA15" s="16"/>
+      <c r="AB15" s="16"/>
+      <c r="AC15" s="16"/>
+      <c r="AD15" s="16"/>
+      <c r="AF15" s="16"/>
+      <c r="AG15" s="16"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C16" s="17"/>
       <c r="D16" s="3" t="str">
         <f t="shared" si="1"/>
         <v>05</v>
@@ -2065,16 +2001,16 @@
       <c r="F16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="16" t="s">
+      <c r="G16" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16" t="s">
+      <c r="H16" s="17"/>
+      <c r="I16" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
       <c r="M16" s="3" t="str">
         <f t="shared" si="2"/>
         <v>05</v>
@@ -2083,8 +2019,8 @@
         <f t="shared" si="0"/>
         <v>gen[5]</v>
       </c>
-      <c r="O16" s="36" t="s">
-        <v>154</v>
+      <c r="O16" s="18" t="s">
+        <v>152</v>
       </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
@@ -2102,9 +2038,9 @@
     </row>
     <row r="17" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B17" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C17" s="17"/>
       <c r="D17" s="3" t="str">
         <f t="shared" si="1"/>
         <v>06</v>
@@ -2119,14 +2055,14 @@
         <v>12</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I17" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I17" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
       <c r="M17" s="3" t="str">
         <f t="shared" si="2"/>
         <v>06</v>
@@ -2135,13 +2071,13 @@
         <f t="shared" ref="N17:N35" si="3">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M17)),"]")</f>
         <v>gen[6]</v>
       </c>
-      <c r="O17" s="36"/>
+      <c r="O17" s="18"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C18" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C18" s="17"/>
       <c r="D18" s="3" t="str">
         <f t="shared" si="1"/>
         <v>07</v>
@@ -2152,16 +2088,16 @@
       <c r="F18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="16" t="s">
+      <c r="G18" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16" t="s">
+      <c r="H18" s="17"/>
+      <c r="I18" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
       <c r="M18" s="3" t="str">
         <f t="shared" si="2"/>
         <v>07</v>
@@ -2170,14 +2106,14 @@
         <f t="shared" si="3"/>
         <v>gen[7]</v>
       </c>
-      <c r="O18" s="36"/>
+      <c r="O18" s="18"/>
       <c r="AE18" s="2"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C19" s="17"/>
       <c r="D19" s="3" t="str">
         <f t="shared" si="1"/>
         <v>08</v>
@@ -2192,14 +2128,14 @@
         <v>12</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I19" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I19" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
       <c r="M19" s="3" t="str">
         <f t="shared" si="2"/>
         <v>08</v>
@@ -2208,14 +2144,14 @@
         <f t="shared" si="3"/>
         <v>gen[8]</v>
       </c>
-      <c r="O19" s="36"/>
+      <c r="O19" s="18"/>
       <c r="V19" s="2"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C20" s="17"/>
       <c r="D20" s="3" t="str">
         <f t="shared" si="1"/>
         <v>09</v>
@@ -2226,16 +2162,16 @@
       <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16" t="s">
+      <c r="H20" s="17"/>
+      <c r="I20" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
       <c r="M20" s="3" t="str">
         <f t="shared" si="2"/>
         <v>09</v>
@@ -2244,15 +2180,15 @@
         <f t="shared" si="3"/>
         <v>gen[9]</v>
       </c>
-      <c r="O20" s="36"/>
+      <c r="O20" s="18"/>
       <c r="R20" s="2"/>
       <c r="V20" s="2"/>
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C21" s="17"/>
       <c r="D21" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0A</v>
@@ -2267,14 +2203,14 @@
         <v>12</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I21" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I21" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
       <c r="M21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0A</v>
@@ -2283,13 +2219,13 @@
         <f t="shared" si="3"/>
         <v>gen[10]</v>
       </c>
-      <c r="O21" s="36"/>
+      <c r="O21" s="18"/>
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C22" s="17"/>
       <c r="D22" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0B</v>
@@ -2300,16 +2236,16 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16" t="s">
+      <c r="H22" s="17"/>
+      <c r="I22" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="17"/>
       <c r="M22" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0B</v>
@@ -2318,7 +2254,7 @@
         <f t="shared" si="3"/>
         <v>gen[11]</v>
       </c>
-      <c r="O22" s="36"/>
+      <c r="O22" s="18"/>
       <c r="S22" s="1"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
@@ -2326,15 +2262,15 @@
     </row>
     <row r="23" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C23" s="17"/>
       <c r="D23" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0C</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
@@ -2343,14 +2279,14 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I23" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
+        <v>92</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
       <c r="M23" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0C</v>
@@ -2359,7 +2295,7 @@
         <f t="shared" si="3"/>
         <v>gen[12]</v>
       </c>
-      <c r="O23" s="36"/>
+      <c r="O23" s="18"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
@@ -2367,29 +2303,29 @@
     </row>
     <row r="24" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B24" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C24" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C24" s="17"/>
       <c r="D24" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0D</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
       <c r="M24" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0D</v>
@@ -2398,21 +2334,21 @@
         <f t="shared" si="3"/>
         <v>gen[13]</v>
       </c>
-      <c r="O24" s="36" t="s">
-        <v>155</v>
+      <c r="O24" s="18" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C25" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C25" s="17"/>
       <c r="D25" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0E</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>11</v>
@@ -2421,14 +2357,14 @@
         <v>12</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I25" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
+        <v>92</v>
+      </c>
+      <c r="I25" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
       <c r="M25" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0E</v>
@@ -2437,33 +2373,33 @@
         <f t="shared" si="3"/>
         <v>gen[14]</v>
       </c>
-      <c r="O25" s="36"/>
+      <c r="O25" s="18"/>
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C26" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C26" s="17"/>
       <c r="D26" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0F</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="16" t="s">
+      <c r="G26" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="J26" s="16"/>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
       <c r="M26" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0F</v>
@@ -2472,19 +2408,19 @@
         <f t="shared" si="3"/>
         <v>gen[15]</v>
       </c>
-      <c r="O26" s="36"/>
+      <c r="O26" s="18"/>
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C27" s="17"/>
       <c r="D27" s="3" t="str">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>11</v>
@@ -2493,14 +2429,14 @@
         <v>12</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I27" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I27" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
       <c r="M27" s="3" t="str">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2509,19 +2445,19 @@
         <f t="shared" si="3"/>
         <v>gen[16]</v>
       </c>
-      <c r="O27" s="36"/>
+      <c r="O27" s="18"/>
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C28" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C28" s="17"/>
       <c r="D28" s="3" t="str">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>11</v>
@@ -2530,14 +2466,14 @@
         <v>12</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
+        <v>92</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="17"/>
       <c r="M28" s="3" t="str">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2546,33 +2482,33 @@
         <f t="shared" si="3"/>
         <v>gen[17]</v>
       </c>
-      <c r="O28" s="36"/>
+      <c r="O28" s="18"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C29" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C29" s="17"/>
       <c r="D29" s="3" t="str">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16" t="s">
+      <c r="H29" s="17"/>
+      <c r="I29" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="17"/>
       <c r="M29" s="3" t="str">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -2581,19 +2517,19 @@
         <f t="shared" si="3"/>
         <v>gen[18]</v>
       </c>
-      <c r="O29" s="36"/>
+      <c r="O29" s="18"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C30" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C30" s="17"/>
       <c r="D30" s="3" t="str">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>11</v>
@@ -2602,14 +2538,14 @@
         <v>12</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I30" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I30" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="17"/>
       <c r="M30" s="3" t="str">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -2618,19 +2554,19 @@
         <f t="shared" si="3"/>
         <v>gen[19]</v>
       </c>
-      <c r="O30" s="36"/>
+      <c r="O30" s="18"/>
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C31" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C31" s="17"/>
       <c r="D31" s="3" t="str">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>11</v>
@@ -2639,14 +2575,14 @@
         <v>12</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I31" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
+        <v>92</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="J31" s="17"/>
+      <c r="K31" s="17"/>
+      <c r="L31" s="17"/>
       <c r="M31" s="3" t="str">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -2655,33 +2591,33 @@
         <f t="shared" si="3"/>
         <v>gen[20]</v>
       </c>
-      <c r="O31" s="36"/>
+      <c r="O31" s="18"/>
     </row>
     <row r="32" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C32" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C32" s="17"/>
       <c r="D32" s="3" t="str">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G32" s="16" t="s">
+      <c r="G32" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16" t="s">
+      <c r="H32" s="17"/>
+      <c r="I32" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17"/>
       <c r="M32" s="3" t="str">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -2690,37 +2626,37 @@
         <f t="shared" si="3"/>
         <v>gen[21]</v>
       </c>
-      <c r="O32" s="36" t="s">
-        <v>156</v>
+      <c r="O32" s="18" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B33" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C33" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C33" s="17"/>
       <c r="D33" s="3" t="str">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="H33" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I33" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="G33" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I33" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+      <c r="L33" s="17"/>
       <c r="M33" s="3" t="str">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -2729,33 +2665,33 @@
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="36"/>
+      <c r="O33" s="18"/>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C34" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C34" s="17"/>
       <c r="D34" s="3" t="str">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="16" t="s">
+      <c r="G34" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="17"/>
       <c r="M34" s="3" t="str">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -2764,44 +2700,44 @@
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="36"/>
+      <c r="O34" s="18"/>
       <c r="R34" t="s">
-        <v>140</v>
-      </c>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
-      <c r="V34" s="28"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
+        <v>138</v>
+      </c>
+      <c r="T34" s="16"/>
+      <c r="U34" s="16"/>
+      <c r="V34" s="16"/>
+      <c r="W34" s="16"/>
+      <c r="X34" s="16"/>
+      <c r="Y34" s="16"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C35" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C35" s="17"/>
       <c r="D35" s="3" t="str">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I35" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
+        <v>92</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="17"/>
       <c r="M35" s="3" t="str">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -2810,55 +2746,55 @@
         <f t="shared" si="3"/>
         <v>gen[24]</v>
       </c>
-      <c r="O35" s="36"/>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
-      <c r="V35" s="28"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
+      <c r="O35" s="18"/>
+      <c r="T35" s="16"/>
+      <c r="U35" s="16"/>
+      <c r="V35" s="16"/>
+      <c r="W35" s="16"/>
+      <c r="X35" s="16"/>
+      <c r="Y35" s="16"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C36" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C36" s="17"/>
       <c r="D36" s="3" t="str">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="16" t="s">
+      <c r="G36" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H36" s="16"/>
-      <c r="I36" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="J36" s="16"/>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
       <c r="M36" s="3" t="str">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
       <c r="N36" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="O36" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B37" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C37" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="17" t="s">
         <v>47</v>
       </c>
       <c r="D37" s="3" t="str">
@@ -2871,17 +2807,17 @@
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="16" t="s">
+      <c r="G37" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H37" s="16"/>
-      <c r="I37" s="16" t="s">
+      <c r="H37" s="17"/>
+      <c r="I37" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="16"/>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16" t="s">
-        <v>106</v>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17" t="s">
+        <v>104</v>
       </c>
       <c r="M37" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2890,35 +2826,35 @@
       <c r="N37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="O37" s="36" t="s">
-        <v>112</v>
+      <c r="O37" s="18" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B38" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C38" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C38" s="17"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1B</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G38" s="16" t="s">
+      <c r="G38" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
       <c r="M38" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1B</v>
@@ -2926,13 +2862,13 @@
       <c r="N38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="36"/>
+      <c r="O38" s="18"/>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C39" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C39" s="17"/>
       <c r="D39" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1C</v>
@@ -2947,14 +2883,14 @@
         <v>12</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I39" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I39" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
       <c r="M39" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1C</v>
@@ -2962,11 +2898,11 @@
       <c r="N39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O39" s="36"/>
+      <c r="O39" s="18"/>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>52</v>
@@ -2976,20 +2912,20 @@
         <v>1D</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F40" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
+        <v>147</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
       <c r="L40" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="M40" s="3" t="str">
         <f t="shared" si="2"/>
@@ -2998,15 +2934,15 @@
       <c r="N40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O40" s="17" t="s">
-        <v>169</v>
+      <c r="O40" s="18" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="41" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B41" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C41" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C41" s="17" t="s">
         <v>3</v>
       </c>
       <c r="D41" s="3" t="str">
@@ -3019,17 +2955,17 @@
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G41" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="H41" s="16"/>
-      <c r="I41" s="16" t="s">
+      <c r="G41" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="H41" s="17"/>
+      <c r="I41" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="J41" s="16"/>
-      <c r="K41" s="16"/>
+      <c r="J41" s="17"/>
+      <c r="K41" s="17"/>
       <c r="L41" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M41" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3043,9 +2979,9 @@
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C42" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C42" s="17"/>
       <c r="D42" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1F</v>
@@ -3056,17 +2992,17 @@
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="H42" s="16"/>
-      <c r="I42" s="16" t="s">
+      <c r="G42" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="H42" s="17"/>
+      <c r="I42" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="J42" s="16"/>
-      <c r="K42" s="16"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="17"/>
       <c r="L42" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M42" s="3" t="str">
         <f t="shared" si="2"/>
@@ -3075,13 +3011,13 @@
       <c r="N42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="19"/>
+      <c r="O42" s="18"/>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C43" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="17" t="s">
         <v>51</v>
       </c>
       <c r="D43" s="3" t="str">
@@ -3094,33 +3030,33 @@
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="16" t="s">
+      <c r="G43" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H43" s="16"/>
-      <c r="I43" s="16" t="s">
+      <c r="H43" s="17"/>
+      <c r="I43" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="J43" s="16"/>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16" t="s">
-        <v>186</v>
+      <c r="J43" s="17"/>
+      <c r="K43" s="17"/>
+      <c r="L43" s="17" t="s">
+        <v>184</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="O43" s="17" t="s">
-        <v>192</v>
+        <v>166</v>
+      </c>
+      <c r="O43" s="18" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C44" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C44" s="17"/>
       <c r="D44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 32))</f>
         <v>40~5F</v>
@@ -3131,30 +3067,30 @@
       <c r="F44" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G44" s="16" t="s">
+      <c r="G44" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H44" s="16"/>
-      <c r="I44" s="16" t="s">
+      <c r="H44" s="17"/>
+      <c r="I44" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="J44" s="16"/>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
+      <c r="J44" s="17"/>
+      <c r="K44" s="17"/>
+      <c r="L44" s="17"/>
       <c r="M44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M43,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M43,"-", -1))+1,"0"))</f>
         <v>ex-2</v>
       </c>
       <c r="N44" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O44" s="18"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C45" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C45" s="17" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="3" t="str">
@@ -3167,64 +3103,64 @@
       <c r="F45" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G45" s="16" t="s">
+      <c r="G45" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H45" s="16"/>
-      <c r="I45" s="16" t="s">
+      <c r="H45" s="17"/>
+      <c r="I45" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="J45" s="16"/>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="17"/>
       <c r="M45" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M44,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M44,"-", -1))+1,"0"))</f>
         <v>ex-3</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="O45" s="18"/>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C46" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C46" s="17"/>
       <c r="D46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 8))</f>
         <v>68~6F</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G46" s="16" t="s">
+      <c r="G46" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H46" s="16"/>
-      <c r="I46" s="16" t="s">
+      <c r="H46" s="17"/>
+      <c r="I46" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="J46" s="16"/>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
+      <c r="L46" s="17"/>
       <c r="M46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M45,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M45,"-", -1))+1,"0"))</f>
         <v>ex-4</v>
       </c>
       <c r="N46" s="3" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="O46" s="18"/>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C47" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C47" s="17"/>
       <c r="D47" s="4" t="str">
         <f>DEC2HEX(HEX2DEC(RIGHT(D46,LEN(D46)-FIND("~",D46,1))) + 1)</f>
         <v>70</v>
@@ -3235,30 +3171,30 @@
       <c r="F47" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G47" s="16" t="s">
+      <c r="G47" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H47" s="16"/>
-      <c r="I47" s="16" t="s">
+      <c r="H47" s="17"/>
+      <c r="I47" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="16"/>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
+      <c r="J47" s="17"/>
+      <c r="K47" s="17"/>
+      <c r="L47" s="17"/>
       <c r="M47" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M46,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M46,"-", -1))+1,"0"))</f>
         <v>ex-5</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="O47" s="19"/>
+        <v>174</v>
+      </c>
+      <c r="O47" s="18"/>
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C48" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C48" s="17"/>
       <c r="D48" s="3" t="str">
         <f t="shared" ref="D48:D54" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D47)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D47)+1))</f>
         <v>71</v>
@@ -3266,128 +3202,128 @@
       <c r="E48" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G48" s="16"/>
-      <c r="H48" s="16"/>
-      <c r="I48" s="16" t="s">
+      <c r="F48" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G48" s="17"/>
+      <c r="H48" s="17"/>
+      <c r="I48" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="J48" s="16"/>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16" t="s">
+      <c r="J48" s="17"/>
+      <c r="K48" s="17"/>
+      <c r="L48" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="M48" s="16"/>
-      <c r="N48" s="16"/>
-      <c r="O48" s="36"/>
+      <c r="M48" s="17"/>
+      <c r="N48" s="17"/>
+      <c r="O48" s="18"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C49" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C49" s="17"/>
       <c r="D49" s="3" t="str">
         <f t="shared" si="5"/>
         <v>72</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F49" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="F49" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G49" s="16"/>
-      <c r="H49" s="16"/>
-      <c r="I49" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="J49" s="16"/>
-      <c r="K49" s="16"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="17"/>
       <c r="L49" s="6" t="s">
         <v>46</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="N49" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="O49" s="36"/>
+        <v>111</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="O49" s="18"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C50" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C50" s="17"/>
       <c r="D50" s="3" t="str">
         <f t="shared" si="5"/>
         <v>73</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="F50" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G50" s="16"/>
-      <c r="H50" s="16"/>
-      <c r="I50" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="J50" s="16"/>
-      <c r="K50" s="16"/>
+        <v>172</v>
+      </c>
+      <c r="F50" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G50" s="17"/>
+      <c r="H50" s="17"/>
+      <c r="I50" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
       <c r="L50" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M50" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N50" s="16" t="s">
+      <c r="N50" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="O50" s="36"/>
+      <c r="O50" s="18"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="C51" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="C51" s="17"/>
       <c r="D51" s="3" t="str">
         <f t="shared" si="5"/>
         <v>74</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="F51" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G51" s="16"/>
-      <c r="H51" s="16"/>
-      <c r="I51" s="16" t="s">
-        <v>172</v>
-      </c>
-      <c r="J51" s="16"/>
-      <c r="K51" s="16"/>
+        <v>171</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G51" s="17"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="J51" s="17"/>
+      <c r="K51" s="17"/>
       <c r="L51" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M51" s="3" t="str">
         <f t="shared" ref="M51:M59" si="6">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M50)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M50)+1))</f>
         <v>01</v>
       </c>
-      <c r="N51" s="16" t="s">
+      <c r="N51" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="O51" s="36"/>
+      <c r="O51" s="18"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C52" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C52" s="17"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="5"/>
         <v>75</v>
@@ -3395,33 +3331,33 @@
       <c r="E52" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F52" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G52" s="16"/>
-      <c r="H52" s="16"/>
-      <c r="I52" s="16" t="s">
+      <c r="F52" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="17"/>
+      <c r="H52" s="17"/>
+      <c r="I52" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="J52" s="16"/>
-      <c r="K52" s="16"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
       <c r="L52" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M52" s="3" t="str">
         <f t="shared" si="6"/>
         <v>02</v>
       </c>
-      <c r="N52" s="16" t="s">
+      <c r="N52" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="O52" s="36"/>
+      <c r="O52" s="18"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C53" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" s="17" t="s">
         <v>50</v>
       </c>
       <c r="D53" s="3" t="str">
@@ -3429,145 +3365,145 @@
         <v>76</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="F53" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G53" s="16"/>
-      <c r="H53" s="16"/>
-      <c r="I53" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="J53" s="16"/>
-      <c r="K53" s="16"/>
+        <v>101</v>
+      </c>
+      <c r="F53" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G53" s="17"/>
+      <c r="H53" s="17"/>
+      <c r="I53" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="J53" s="17"/>
+      <c r="K53" s="17"/>
       <c r="L53" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M53" s="3" t="str">
         <f t="shared" si="6"/>
         <v>03</v>
       </c>
-      <c r="N53" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="O53" s="36"/>
+      <c r="N53" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="O53" s="18"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C54" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C54" s="17"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="5"/>
         <v>77</v>
       </c>
       <c r="E54" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F54" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G54" s="17"/>
+      <c r="H54" s="17"/>
+      <c r="I54" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="F54" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G54" s="16"/>
-      <c r="H54" s="16"/>
-      <c r="I54" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="J54" s="16"/>
-      <c r="K54" s="16"/>
+      <c r="J54" s="17"/>
+      <c r="K54" s="17"/>
       <c r="L54" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M54" s="3" t="str">
         <f t="shared" si="6"/>
         <v>04</v>
       </c>
-      <c r="N54" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="O54" s="36"/>
+      <c r="N54" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="O54" s="18"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C55" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C55" s="17"/>
       <c r="D55" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="I55" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="J55" s="16"/>
-      <c r="K55" s="16"/>
+      <c r="I55" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="J55" s="17"/>
+      <c r="K55" s="17"/>
       <c r="L55" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M55" s="3" t="str">
         <f t="shared" si="6"/>
         <v>05</v>
       </c>
-      <c r="N55" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="O55" s="36"/>
+      <c r="N55" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="O55" s="18"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C56" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C56" s="17"/>
       <c r="D56" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D55)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D55)+1))</f>
         <v>79</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="I56" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="J56" s="16"/>
-      <c r="K56" s="16"/>
+        <v>159</v>
+      </c>
+      <c r="I56" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="J56" s="17"/>
+      <c r="K56" s="17"/>
       <c r="L56" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="M56" s="3" t="str">
         <f t="shared" si="6"/>
         <v>06</v>
       </c>
-      <c r="N56" s="16" t="s">
+      <c r="N56" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="O56" s="36"/>
+      <c r="O56" s="18"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C57" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C57" s="17" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="3" t="str">
@@ -3575,77 +3511,77 @@
         <v>7A</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="I57" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="J57" s="16"/>
-      <c r="K57" s="16"/>
+        <v>200</v>
+      </c>
+      <c r="I57" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="J57" s="17"/>
+      <c r="K57" s="17"/>
       <c r="L57" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M57" s="3" t="str">
         <f t="shared" si="6"/>
         <v>07</v>
       </c>
-      <c r="N57" s="16" t="s">
+      <c r="N57" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="O57" s="36"/>
+      <c r="O57" s="18"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C58" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C58" s="17"/>
       <c r="D58" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D57)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D57)+1))</f>
         <v>7B</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="I58" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="J58" s="16"/>
-      <c r="K58" s="16"/>
+        <v>200</v>
+      </c>
+      <c r="I58" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="J58" s="17"/>
+      <c r="K58" s="17"/>
       <c r="L58" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M58" s="3" t="str">
         <f t="shared" si="6"/>
         <v>08</v>
       </c>
-      <c r="N58" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="O58" s="36"/>
+      <c r="N58" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="O58" s="18"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C59" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C59" s="17" t="s">
         <v>38</v>
       </c>
       <c r="D59" s="3" t="str">
@@ -3653,75 +3589,75 @@
         <v>7C</v>
       </c>
       <c r="E59" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F59" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G59" s="17"/>
+      <c r="H59" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="I59" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="F59" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G59" s="16"/>
-      <c r="H59" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="I59" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="J59" s="16"/>
-      <c r="K59" s="16"/>
+      <c r="J59" s="17"/>
+      <c r="K59" s="17"/>
       <c r="L59" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="M59" s="3" t="str">
         <f t="shared" si="6"/>
         <v>09</v>
       </c>
-      <c r="N59" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="O59" s="36"/>
+      <c r="N59" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="O59" s="18"/>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C60" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C60" s="17"/>
       <c r="D60" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7D</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F60" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="H60" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="G60" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="H60" s="3" t="s">
+      <c r="I60" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="I60" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="J60" s="16"/>
-      <c r="K60" s="16"/>
+      <c r="J60" s="17"/>
+      <c r="K60" s="17"/>
       <c r="L60" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M60" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M59) + 1),"~",DEC2HEX(HEX2DEC(M59) + 6))</f>
         <v>A~F</v>
       </c>
-      <c r="N60" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="O60" s="36"/>
+      <c r="N60" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="O60" s="18"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B61" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C61" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C61" s="5" t="s">
         <v>82</v>
       </c>
       <c r="D61" s="3" t="str">
@@ -3729,119 +3665,126 @@
         <v>7E</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="G61" s="15" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="I61" s="16" t="s">
-        <v>206</v>
-      </c>
-      <c r="J61" s="16"/>
-      <c r="K61" s="16"/>
+        <v>175</v>
+      </c>
+      <c r="I61" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="J61" s="17"/>
+      <c r="K61" s="17"/>
       <c r="L61" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M61" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(M60,LEN(M60)-FIND("~",M60,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(M60,LEN(M60)-FIND("~",M60,1))) + 16))</f>
         <v>10~1F</v>
       </c>
-      <c r="N61" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="O61" s="36"/>
+      <c r="N61" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="O61" s="18"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C62" s="16"/>
+        <v>90</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>205</v>
+      </c>
       <c r="D62" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7F</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>179</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="F62" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="G62" s="17"/>
       <c r="H62" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="I62" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="J62" s="16"/>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="M62" s="16"/>
-      <c r="N62" s="16"/>
-      <c r="O62" s="36"/>
+        <v>206</v>
+      </c>
+      <c r="I62" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="J62" s="17"/>
+      <c r="K62" s="17"/>
+      <c r="L62" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="M62" s="17"/>
+      <c r="N62" s="17"/>
+      <c r="O62" s="18"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D63" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(D62) + 1),"~","FF")</f>
         <v>80~FF</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F63" s="20" t="s">
-        <v>94</v>
-      </c>
-      <c r="G63" s="21"/>
-      <c r="H63" s="22"/>
-      <c r="I63" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="J63" s="21"/>
-      <c r="K63" s="22"/>
+        <v>84</v>
+      </c>
+      <c r="F63" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G63" s="17"/>
+      <c r="H63" s="17"/>
+      <c r="I63" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="J63" s="17"/>
+      <c r="K63" s="17"/>
       <c r="L63" s="5" t="s">
         <v>39</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N63" s="5" t="s">
         <v>39</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="24"/>
-      <c r="C64" s="25"/>
-      <c r="D64" s="25"/>
-      <c r="E64" s="25"/>
-      <c r="F64" s="25"/>
-      <c r="G64" s="26"/>
-      <c r="H64" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="I64" s="21"/>
-      <c r="J64" s="21"/>
-      <c r="K64" s="23"/>
+      <c r="B64" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="C64" s="3" t="str">
+        <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M47,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M47,"-", -1))+1,"0"))</f>
+        <v>ex-6</v>
+      </c>
+      <c r="D64" s="32"/>
+      <c r="E64" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="F64" s="41"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="I64" s="17"/>
+      <c r="J64" s="17"/>
+      <c r="K64" s="17"/>
       <c r="L64" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="M64" s="7" t="s">
         <v>27</v>
@@ -3851,27 +3794,30 @@
         <v>4</v>
       </c>
       <c r="O64" s="11" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="27"/>
-      <c r="C65" s="28"/>
-      <c r="D65" s="28"/>
-      <c r="E65" s="28"/>
-      <c r="F65" s="28"/>
-      <c r="G65" s="29"/>
+      <c r="B65" s="35"/>
+      <c r="C65" s="3" t="str">
+        <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(C64,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(C64,"-", -1))+1,"0"))</f>
+        <v>ex-7</v>
+      </c>
+      <c r="D65" s="32"/>
+      <c r="E65" s="39"/>
+      <c r="F65" s="42"/>
+      <c r="G65" s="30"/>
       <c r="H65" s="4" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="L65" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L64+1)</f>
@@ -3885,27 +3831,30 @@
         <v>5</v>
       </c>
       <c r="O65" s="11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="27"/>
-      <c r="C66" s="28"/>
-      <c r="D66" s="28"/>
-      <c r="E66" s="28"/>
-      <c r="F66" s="28"/>
-      <c r="G66" s="29"/>
+      <c r="B66" s="35"/>
+      <c r="C66" s="3" t="str">
+        <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(C65,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(C65,"-", -1))+1,"0"))</f>
+        <v>ex-8</v>
+      </c>
+      <c r="D66" s="32"/>
+      <c r="E66" s="39"/>
+      <c r="F66" s="42"/>
+      <c r="G66" s="30"/>
       <c r="H66" s="3" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="L66" s="3" t="str">
         <f>_xlfn.VALUETOTEXT(L65+1)</f>
@@ -3919,22 +3868,25 @@
         <v>6</v>
       </c>
       <c r="O66" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="67" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="30"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="31"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="32"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="34" t="str">
+        <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(C66,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(C66,"-", -1))+1,"0"))</f>
+        <v>ex-9</v>
+      </c>
+      <c r="D67" s="34"/>
+      <c r="E67" s="40"/>
+      <c r="F67" s="43"/>
+      <c r="G67" s="31"/>
       <c r="H67" s="33" t="s">
-        <v>204</v>
-      </c>
-      <c r="I67" s="34"/>
-      <c r="J67" s="34"/>
-      <c r="K67" s="35"/>
+        <v>201</v>
+      </c>
+      <c r="I67" s="33"/>
+      <c r="J67" s="33"/>
+      <c r="K67" s="33"/>
       <c r="L67" s="12" t="str">
         <f>_xlfn.VALUETOTEXT(L66+1)</f>
         <v>3</v>
@@ -3947,11 +3899,120 @@
         <v>7</v>
       </c>
       <c r="O67" s="14" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="131">
+  <mergeCells count="133">
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="E64:E67"/>
+    <mergeCell ref="F64:G67"/>
+    <mergeCell ref="L43:L47"/>
+    <mergeCell ref="I61:K61"/>
+    <mergeCell ref="I62:K62"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="O40:O42"/>
+    <mergeCell ref="O43:O47"/>
+    <mergeCell ref="F63:H63"/>
+    <mergeCell ref="I63:K63"/>
+    <mergeCell ref="N55:O55"/>
+    <mergeCell ref="N61:O61"/>
+    <mergeCell ref="N58:O58"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="I59:K59"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="L62:O62"/>
+    <mergeCell ref="F54:H54"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="F53:H53"/>
+    <mergeCell ref="C53:C56"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="H64:K64"/>
+    <mergeCell ref="H67:K67"/>
+    <mergeCell ref="O12:O15"/>
+    <mergeCell ref="O32:O35"/>
+    <mergeCell ref="O37:O39"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="O16:O23"/>
+    <mergeCell ref="O24:O31"/>
+    <mergeCell ref="L11:L36"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="C45:C52"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
     <mergeCell ref="AF15:AG15"/>
     <mergeCell ref="L48:O48"/>
     <mergeCell ref="AC15:AD15"/>
@@ -3976,113 +4037,6 @@
     <mergeCell ref="F50:H50"/>
     <mergeCell ref="F52:H52"/>
     <mergeCell ref="I52:K52"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="C45:C52"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="O16:O23"/>
-    <mergeCell ref="O24:O31"/>
-    <mergeCell ref="L11:L36"/>
-    <mergeCell ref="H64:K64"/>
-    <mergeCell ref="B64:G67"/>
-    <mergeCell ref="H67:K67"/>
-    <mergeCell ref="O12:O15"/>
-    <mergeCell ref="O32:O35"/>
-    <mergeCell ref="O37:O39"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N54:O54"/>
-    <mergeCell ref="L43:L47"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="O40:O42"/>
-    <mergeCell ref="O43:O47"/>
-    <mergeCell ref="F63:H63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="N55:O55"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="N58:O58"/>
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="N60:O60"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="L62:O62"/>
-    <mergeCell ref="F54:H54"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="C53:C56"/>
-    <mergeCell ref="C57:C58"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: bootloader, byte addressed strings, move emulator to tools
- boot/src/boot.asm: copy ROM program (dlnk header) to RAM and jump
- fix rom-test ld wiring and BTB taken-branch target+4 fetch
- dlnk 8 byte header (start, length), -raw, -start; _start in entry programs
- io / floatingpoint / calc / picalc: byte strings, little endian
- emulator moved to tools/emu/isa32emu.py (little endian, byte memory)
- archive old program/*.txt into program/archive
- todo.md: progress as of 2026-10-17

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QJGhBeyFbVexj3aLG7xNkt
</commit_message>
<xml_diff>
--- a/ISA-32.xlsx
+++ b/ISA-32.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\taeh5\Homemade Computer\computer 32 (new)\digital computer 32\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A77CC6D-249D-47F7-835D-0D6500569CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5490EDAD-AB23-4D54-874A-53F91A8A842B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8114D55D-0332-45B3-9181-1200CCB278EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1197,7 +1197,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1246,88 +1246,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1676,74 +1670,74 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="22"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="33"/>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B7" s="23"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="25"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
+      <c r="K7" s="35"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="35"/>
+      <c r="N7" s="35"/>
+      <c r="O7" s="36"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B8" s="26"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="27"/>
-      <c r="M8" s="27"/>
-      <c r="N8" s="27"/>
-      <c r="O8" s="28"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
+      <c r="N8" s="38"/>
+      <c r="O8" s="39"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17" t="s">
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="18"/>
+      <c r="M9" s="28"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="29"/>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="9" t="s">
@@ -1767,11 +1761,11 @@
       <c r="H10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="I10" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
       <c r="L10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1789,7 +1783,7 @@
       <c r="B11" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="28" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1807,12 +1801,12 @@
       <c r="H11" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I11" s="17" t="s">
+      <c r="I11" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17" t="s">
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28" t="s">
         <v>103</v>
       </c>
       <c r="M11" s="4" t="s">
@@ -1830,7 +1824,7 @@
       <c r="B12" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C12" s="17"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="3" t="str">
         <f t="shared" ref="D12:D36" si="1">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D11)+1))</f>
         <v>01</v>
@@ -1847,12 +1841,12 @@
       <c r="H12" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I12" s="17" t="s">
+      <c r="I12" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="28"/>
+      <c r="L12" s="28"/>
       <c r="M12" s="3" t="str">
         <f t="shared" ref="M12:M42" si="2">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M11)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M11)+1))</f>
         <v>01</v>
@@ -1861,7 +1855,7 @@
         <f t="shared" si="0"/>
         <v>gen[1]</v>
       </c>
-      <c r="O12" s="18" t="s">
+      <c r="O12" s="29" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1869,7 +1863,7 @@
       <c r="B13" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="17"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="3" t="str">
         <f t="shared" si="1"/>
         <v>02</v>
@@ -1880,16 +1874,16 @@
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17" t="s">
+      <c r="H13" s="28"/>
+      <c r="I13" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
       <c r="M13" s="3" t="str">
         <f t="shared" si="2"/>
         <v>02</v>
@@ -1898,13 +1892,13 @@
         <f t="shared" si="0"/>
         <v>gen[2]</v>
       </c>
-      <c r="O13" s="18"/>
+      <c r="O13" s="29"/>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="17"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="3" t="str">
         <f t="shared" si="1"/>
         <v>03</v>
@@ -1921,12 +1915,12 @@
       <c r="H14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="I14" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="28"/>
+      <c r="L14" s="28"/>
       <c r="M14" s="3" t="str">
         <f t="shared" si="2"/>
         <v>03</v>
@@ -1935,13 +1929,13 @@
         <f t="shared" si="0"/>
         <v>gen[3]</v>
       </c>
-      <c r="O14" s="18"/>
+      <c r="O14" s="29"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C15" s="17"/>
+      <c r="C15" s="28"/>
       <c r="D15" s="3" t="str">
         <f t="shared" si="1"/>
         <v>04</v>
@@ -1958,12 +1952,12 @@
       <c r="H15" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="I15" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="28"/>
       <c r="M15" s="3" t="str">
         <f t="shared" si="2"/>
         <v>04</v>
@@ -1972,25 +1966,25 @@
         <f t="shared" si="0"/>
         <v>gen[4]</v>
       </c>
-      <c r="O15" s="18"/>
-      <c r="U15" s="16"/>
-      <c r="V15" s="16"/>
-      <c r="W15" s="16"/>
-      <c r="X15" s="16"/>
-      <c r="Y15" s="16"/>
-      <c r="Z15" s="16"/>
-      <c r="AA15" s="16"/>
-      <c r="AB15" s="16"/>
-      <c r="AC15" s="16"/>
-      <c r="AD15" s="16"/>
-      <c r="AF15" s="16"/>
-      <c r="AG15" s="16"/>
+      <c r="O15" s="29"/>
+      <c r="U15" s="40"/>
+      <c r="V15" s="40"/>
+      <c r="W15" s="40"/>
+      <c r="X15" s="40"/>
+      <c r="Y15" s="40"/>
+      <c r="Z15" s="40"/>
+      <c r="AA15" s="40"/>
+      <c r="AB15" s="40"/>
+      <c r="AC15" s="40"/>
+      <c r="AD15" s="40"/>
+      <c r="AF15" s="40"/>
+      <c r="AG15" s="40"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="17"/>
+      <c r="C16" s="28"/>
       <c r="D16" s="3" t="str">
         <f t="shared" si="1"/>
         <v>05</v>
@@ -2001,16 +1995,16 @@
       <c r="F16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="G16" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17" t="s">
+      <c r="H16" s="28"/>
+      <c r="I16" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
       <c r="M16" s="3" t="str">
         <f t="shared" si="2"/>
         <v>05</v>
@@ -2019,7 +2013,7 @@
         <f t="shared" si="0"/>
         <v>gen[5]</v>
       </c>
-      <c r="O16" s="18" t="s">
+      <c r="O16" s="29" t="s">
         <v>152</v>
       </c>
       <c r="U16" s="2"/>
@@ -2040,7 +2034,7 @@
       <c r="B17" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="17"/>
+      <c r="C17" s="28"/>
       <c r="D17" s="3" t="str">
         <f t="shared" si="1"/>
         <v>06</v>
@@ -2057,12 +2051,12 @@
       <c r="H17" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I17" s="17" t="s">
+      <c r="I17" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
+      <c r="J17" s="28"/>
+      <c r="K17" s="28"/>
+      <c r="L17" s="28"/>
       <c r="M17" s="3" t="str">
         <f t="shared" si="2"/>
         <v>06</v>
@@ -2071,13 +2065,13 @@
         <f t="shared" ref="N17:N35" si="3">_xlfn.TEXTJOIN(,TRUE,"gen[",_xlfn.VALUETOTEXT(HEX2DEC(M17)),"]")</f>
         <v>gen[6]</v>
       </c>
-      <c r="O17" s="18"/>
+      <c r="O17" s="29"/>
     </row>
     <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="17"/>
+      <c r="C18" s="28"/>
       <c r="D18" s="3" t="str">
         <f t="shared" si="1"/>
         <v>07</v>
@@ -2088,16 +2082,16 @@
       <c r="F18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="17" t="s">
+      <c r="G18" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17" t="s">
+      <c r="H18" s="28"/>
+      <c r="I18" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
       <c r="M18" s="3" t="str">
         <f t="shared" si="2"/>
         <v>07</v>
@@ -2106,14 +2100,14 @@
         <f t="shared" si="3"/>
         <v>gen[7]</v>
       </c>
-      <c r="O18" s="18"/>
+      <c r="O18" s="29"/>
       <c r="AE18" s="2"/>
     </row>
     <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="17"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="3" t="str">
         <f t="shared" si="1"/>
         <v>08</v>
@@ -2130,12 +2124,12 @@
       <c r="H19" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I19" s="17" t="s">
+      <c r="I19" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="28"/>
+      <c r="L19" s="28"/>
       <c r="M19" s="3" t="str">
         <f t="shared" si="2"/>
         <v>08</v>
@@ -2144,14 +2138,14 @@
         <f t="shared" si="3"/>
         <v>gen[8]</v>
       </c>
-      <c r="O19" s="18"/>
+      <c r="O19" s="29"/>
       <c r="V19" s="2"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="17"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="3" t="str">
         <f t="shared" si="1"/>
         <v>09</v>
@@ -2162,16 +2156,16 @@
       <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="G20" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17" t="s">
+      <c r="H20" s="28"/>
+      <c r="I20" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="28"/>
+      <c r="L20" s="28"/>
       <c r="M20" s="3" t="str">
         <f t="shared" si="2"/>
         <v>09</v>
@@ -2180,7 +2174,7 @@
         <f t="shared" si="3"/>
         <v>gen[9]</v>
       </c>
-      <c r="O20" s="18"/>
+      <c r="O20" s="29"/>
       <c r="R20" s="2"/>
       <c r="V20" s="2"/>
     </row>
@@ -2188,7 +2182,7 @@
       <c r="B21" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="17"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0A</v>
@@ -2205,12 +2199,12 @@
       <c r="H21" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I21" s="17" t="s">
+      <c r="I21" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
+      <c r="J21" s="28"/>
+      <c r="K21" s="28"/>
+      <c r="L21" s="28"/>
       <c r="M21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0A</v>
@@ -2219,13 +2213,13 @@
         <f t="shared" si="3"/>
         <v>gen[10]</v>
       </c>
-      <c r="O21" s="18"/>
+      <c r="O21" s="29"/>
     </row>
     <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="17"/>
+      <c r="C22" s="28"/>
       <c r="D22" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0B</v>
@@ -2236,16 +2230,16 @@
       <c r="F22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="17" t="s">
+      <c r="G22" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17" t="s">
+      <c r="H22" s="28"/>
+      <c r="I22" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
+      <c r="J22" s="28"/>
+      <c r="K22" s="28"/>
+      <c r="L22" s="28"/>
       <c r="M22" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0B</v>
@@ -2254,7 +2248,7 @@
         <f t="shared" si="3"/>
         <v>gen[11]</v>
       </c>
-      <c r="O22" s="18"/>
+      <c r="O22" s="29"/>
       <c r="S22" s="1"/>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
@@ -2264,7 +2258,7 @@
       <c r="B23" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="17"/>
+      <c r="C23" s="28"/>
       <c r="D23" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0C</v>
@@ -2281,12 +2275,12 @@
       <c r="H23" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I23" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
+      <c r="I23" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="J23" s="28"/>
+      <c r="K23" s="28"/>
+      <c r="L23" s="28"/>
       <c r="M23" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0C</v>
@@ -2295,7 +2289,7 @@
         <f t="shared" si="3"/>
         <v>gen[12]</v>
       </c>
-      <c r="O23" s="18"/>
+      <c r="O23" s="29"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
@@ -2305,7 +2299,7 @@
       <c r="B24" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="17"/>
+      <c r="C24" s="28"/>
       <c r="D24" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0D</v>
@@ -2316,16 +2310,16 @@
       <c r="F24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="G24" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="17"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="J24" s="28"/>
+      <c r="K24" s="28"/>
+      <c r="L24" s="28"/>
       <c r="M24" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0D</v>
@@ -2334,7 +2328,7 @@
         <f t="shared" si="3"/>
         <v>gen[13]</v>
       </c>
-      <c r="O24" s="18" t="s">
+      <c r="O24" s="29" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2342,7 +2336,7 @@
       <c r="B25" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C25" s="17"/>
+      <c r="C25" s="28"/>
       <c r="D25" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0E</v>
@@ -2359,12 +2353,12 @@
       <c r="H25" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I25" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="17"/>
+      <c r="I25" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="J25" s="28"/>
+      <c r="K25" s="28"/>
+      <c r="L25" s="28"/>
       <c r="M25" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0E</v>
@@ -2373,13 +2367,13 @@
         <f t="shared" si="3"/>
         <v>gen[14]</v>
       </c>
-      <c r="O25" s="18"/>
+      <c r="O25" s="29"/>
     </row>
     <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="17"/>
+      <c r="C26" s="28"/>
       <c r="D26" s="3" t="str">
         <f t="shared" si="1"/>
         <v>0F</v>
@@ -2390,16 +2384,16 @@
       <c r="F26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28" t="s">
+        <v>136</v>
+      </c>
+      <c r="J26" s="28"/>
+      <c r="K26" s="28"/>
+      <c r="L26" s="28"/>
       <c r="M26" s="3" t="str">
         <f t="shared" si="2"/>
         <v>0F</v>
@@ -2408,13 +2402,13 @@
         <f t="shared" si="3"/>
         <v>gen[15]</v>
       </c>
-      <c r="O26" s="18"/>
+      <c r="O26" s="29"/>
     </row>
     <row r="27" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C27" s="17"/>
+      <c r="C27" s="28"/>
       <c r="D27" s="3" t="str">
         <f t="shared" si="1"/>
         <v>10</v>
@@ -2431,12 +2425,12 @@
       <c r="H27" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I27" s="17" t="s">
+      <c r="I27" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="J27" s="17"/>
-      <c r="K27" s="17"/>
-      <c r="L27" s="17"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="28"/>
+      <c r="L27" s="28"/>
       <c r="M27" s="3" t="str">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -2445,13 +2439,13 @@
         <f t="shared" si="3"/>
         <v>gen[16]</v>
       </c>
-      <c r="O27" s="18"/>
+      <c r="O27" s="29"/>
     </row>
     <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="17"/>
+      <c r="C28" s="28"/>
       <c r="D28" s="3" t="str">
         <f t="shared" si="1"/>
         <v>11</v>
@@ -2468,12 +2462,12 @@
       <c r="H28" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I28" s="17" t="s">
+      <c r="I28" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="J28" s="17"/>
-      <c r="K28" s="17"/>
-      <c r="L28" s="17"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
       <c r="M28" s="3" t="str">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -2482,13 +2476,13 @@
         <f t="shared" si="3"/>
         <v>gen[17]</v>
       </c>
-      <c r="O28" s="18"/>
+      <c r="O28" s="29"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B29" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="17"/>
+      <c r="C29" s="28"/>
       <c r="D29" s="3" t="str">
         <f t="shared" si="1"/>
         <v>12</v>
@@ -2499,16 +2493,16 @@
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17" t="s">
+      <c r="H29" s="28"/>
+      <c r="I29" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="17"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
       <c r="M29" s="3" t="str">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -2517,13 +2511,13 @@
         <f t="shared" si="3"/>
         <v>gen[18]</v>
       </c>
-      <c r="O29" s="18"/>
+      <c r="O29" s="29"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B30" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C30" s="17"/>
+      <c r="C30" s="28"/>
       <c r="D30" s="3" t="str">
         <f t="shared" si="1"/>
         <v>13</v>
@@ -2540,12 +2534,12 @@
       <c r="H30" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I30" s="17" t="s">
+      <c r="I30" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
       <c r="M30" s="3" t="str">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -2554,13 +2548,13 @@
         <f t="shared" si="3"/>
         <v>gen[19]</v>
       </c>
-      <c r="O30" s="18"/>
+      <c r="O30" s="29"/>
     </row>
     <row r="31" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B31" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C31" s="17"/>
+      <c r="C31" s="28"/>
       <c r="D31" s="3" t="str">
         <f t="shared" si="1"/>
         <v>14</v>
@@ -2577,12 +2571,12 @@
       <c r="H31" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I31" s="17" t="s">
+      <c r="I31" s="28" t="s">
         <v>126</v>
       </c>
-      <c r="J31" s="17"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="28"/>
+      <c r="L31" s="28"/>
       <c r="M31" s="3" t="str">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -2591,13 +2585,13 @@
         <f t="shared" si="3"/>
         <v>gen[20]</v>
       </c>
-      <c r="O31" s="18"/>
+      <c r="O31" s="29"/>
     </row>
     <row r="32" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B32" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C32" s="17"/>
+      <c r="C32" s="28"/>
       <c r="D32" s="3" t="str">
         <f t="shared" si="1"/>
         <v>15</v>
@@ -2608,16 +2602,16 @@
       <c r="F32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G32" s="17" t="s">
+      <c r="G32" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17" t="s">
+      <c r="H32" s="28"/>
+      <c r="I32" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="J32" s="17"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="17"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="28"/>
+      <c r="L32" s="28"/>
       <c r="M32" s="3" t="str">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -2626,7 +2620,7 @@
         <f t="shared" si="3"/>
         <v>gen[21]</v>
       </c>
-      <c r="O32" s="18" t="s">
+      <c r="O32" s="29" t="s">
         <v>154</v>
       </c>
     </row>
@@ -2634,7 +2628,7 @@
       <c r="B33" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="17"/>
+      <c r="C33" s="28"/>
       <c r="D33" s="3" t="str">
         <f t="shared" si="1"/>
         <v>16</v>
@@ -2651,12 +2645,12 @@
       <c r="H33" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I33" s="17" t="s">
+      <c r="I33" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="28"/>
+      <c r="L33" s="28"/>
       <c r="M33" s="3" t="str">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -2665,13 +2659,13 @@
         <f t="shared" si="3"/>
         <v>gen[22]</v>
       </c>
-      <c r="O33" s="18"/>
+      <c r="O33" s="29"/>
     </row>
     <row r="34" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B34" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="17"/>
+      <c r="C34" s="28"/>
       <c r="D34" s="3" t="str">
         <f t="shared" si="1"/>
         <v>17</v>
@@ -2682,16 +2676,16 @@
       <c r="F34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="17" t="s">
+      <c r="G34" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17" t="s">
+      <c r="H34" s="28"/>
+      <c r="I34" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="J34" s="17"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="17"/>
+      <c r="J34" s="28"/>
+      <c r="K34" s="28"/>
+      <c r="L34" s="28"/>
       <c r="M34" s="3" t="str">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -2700,22 +2694,22 @@
         <f t="shared" si="3"/>
         <v>gen[23]</v>
       </c>
-      <c r="O34" s="18"/>
+      <c r="O34" s="29"/>
       <c r="R34" t="s">
         <v>138</v>
       </c>
-      <c r="T34" s="16"/>
-      <c r="U34" s="16"/>
-      <c r="V34" s="16"/>
-      <c r="W34" s="16"/>
-      <c r="X34" s="16"/>
-      <c r="Y34" s="16"/>
+      <c r="T34" s="40"/>
+      <c r="U34" s="40"/>
+      <c r="V34" s="40"/>
+      <c r="W34" s="40"/>
+      <c r="X34" s="40"/>
+      <c r="Y34" s="40"/>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B35" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C35" s="17"/>
+      <c r="C35" s="28"/>
       <c r="D35" s="3" t="str">
         <f t="shared" si="1"/>
         <v>18</v>
@@ -2732,12 +2726,12 @@
       <c r="H35" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I35" s="17" t="s">
+      <c r="I35" s="28" t="s">
         <v>131</v>
       </c>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="17"/>
+      <c r="J35" s="28"/>
+      <c r="K35" s="28"/>
+      <c r="L35" s="28"/>
       <c r="M35" s="3" t="str">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -2746,19 +2740,19 @@
         <f t="shared" si="3"/>
         <v>gen[24]</v>
       </c>
-      <c r="O35" s="18"/>
-      <c r="T35" s="16"/>
-      <c r="U35" s="16"/>
-      <c r="V35" s="16"/>
-      <c r="W35" s="16"/>
-      <c r="X35" s="16"/>
-      <c r="Y35" s="16"/>
+      <c r="O35" s="29"/>
+      <c r="T35" s="40"/>
+      <c r="U35" s="40"/>
+      <c r="V35" s="40"/>
+      <c r="W35" s="40"/>
+      <c r="X35" s="40"/>
+      <c r="Y35" s="40"/>
     </row>
     <row r="36" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B36" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="17"/>
+      <c r="C36" s="28"/>
       <c r="D36" s="3" t="str">
         <f t="shared" si="1"/>
         <v>19</v>
@@ -2769,16 +2763,16 @@
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="17" t="s">
+      <c r="G36" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17" t="s">
+      <c r="H36" s="28"/>
+      <c r="I36" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="28"/>
       <c r="M36" s="3" t="str">
         <f t="shared" si="2"/>
         <v>19</v>
@@ -2794,7 +2788,7 @@
       <c r="B37" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="28" t="s">
         <v>47</v>
       </c>
       <c r="D37" s="3" t="str">
@@ -2807,16 +2801,16 @@
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="17" t="s">
+      <c r="G37" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H37" s="17"/>
-      <c r="I37" s="17" t="s">
+      <c r="H37" s="28"/>
+      <c r="I37" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="J37" s="17"/>
-      <c r="K37" s="17"/>
-      <c r="L37" s="17" t="s">
+      <c r="J37" s="28"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28" t="s">
         <v>104</v>
       </c>
       <c r="M37" s="3" t="str">
@@ -2826,7 +2820,7 @@
       <c r="N37" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="O37" s="18" t="s">
+      <c r="O37" s="29" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2834,7 +2828,7 @@
       <c r="B38" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="17"/>
+      <c r="C38" s="28"/>
       <c r="D38" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1B</v>
@@ -2845,16 +2839,16 @@
       <c r="F38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G38" s="17" t="s">
+      <c r="G38" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17" t="s">
+      <c r="H38" s="28"/>
+      <c r="I38" s="28" t="s">
         <v>142</v>
       </c>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="28"/>
       <c r="M38" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1B</v>
@@ -2862,13 +2856,13 @@
       <c r="N38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="O38" s="18"/>
+      <c r="O38" s="29"/>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B39" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C39" s="17"/>
+      <c r="C39" s="28"/>
       <c r="D39" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1C</v>
@@ -2885,12 +2879,12 @@
       <c r="H39" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I39" s="17" t="s">
+      <c r="I39" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
+      <c r="J39" s="28"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="28"/>
       <c r="M39" s="3" t="str">
         <f t="shared" si="2"/>
         <v>1C</v>
@@ -2898,7 +2892,7 @@
       <c r="N39" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O39" s="18"/>
+      <c r="O39" s="29"/>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B40" s="9" t="s">
@@ -2914,16 +2908,16 @@
       <c r="E40" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="F40" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G40" s="17"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17" t="s">
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="28"/>
       <c r="L40" s="5" t="s">
         <v>105</v>
       </c>
@@ -2934,7 +2928,7 @@
       <c r="N40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O40" s="18" t="s">
+      <c r="O40" s="29" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2942,7 +2936,7 @@
       <c r="B41" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="28" t="s">
         <v>3</v>
       </c>
       <c r="D41" s="3" t="str">
@@ -2955,15 +2949,15 @@
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G41" s="17" t="s">
+      <c r="G41" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17" t="s">
+      <c r="H41" s="28"/>
+      <c r="I41" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="J41" s="17"/>
-      <c r="K41" s="17"/>
+      <c r="J41" s="28"/>
+      <c r="K41" s="28"/>
       <c r="L41" s="5" t="s">
         <v>106</v>
       </c>
@@ -2974,14 +2968,14 @@
       <c r="N41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="O41" s="18"/>
+      <c r="O41" s="29"/>
       <c r="T41" s="2"/>
     </row>
     <row r="42" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B42" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C42" s="17"/>
+      <c r="C42" s="28"/>
       <c r="D42" s="3" t="str">
         <f t="shared" si="4"/>
         <v>1F</v>
@@ -2992,15 +2986,15 @@
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G42" s="17" t="s">
+      <c r="G42" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17" t="s">
+      <c r="H42" s="28"/>
+      <c r="I42" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J42" s="17"/>
-      <c r="K42" s="17"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="28"/>
       <c r="L42" s="5" t="s">
         <v>106</v>
       </c>
@@ -3011,13 +3005,13 @@
       <c r="N42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="18"/>
+      <c r="O42" s="29"/>
     </row>
     <row r="43" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B43" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="C43" s="28" t="s">
         <v>51</v>
       </c>
       <c r="D43" s="3" t="str">
@@ -3030,16 +3024,16 @@
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="17" t="s">
+      <c r="G43" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17" t="s">
+      <c r="H43" s="28"/>
+      <c r="I43" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17" t="s">
+      <c r="J43" s="28"/>
+      <c r="K43" s="28"/>
+      <c r="L43" s="28" t="s">
         <v>184</v>
       </c>
       <c r="M43" s="4" t="s">
@@ -3048,7 +3042,7 @@
       <c r="N43" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="O43" s="18" t="s">
+      <c r="O43" s="29" t="s">
         <v>190</v>
       </c>
     </row>
@@ -3056,7 +3050,7 @@
       <c r="B44" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C44" s="17"/>
+      <c r="C44" s="28"/>
       <c r="D44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D43,LEN(D43)-FIND("~",D43,1))) + 32))</f>
         <v>40~5F</v>
@@ -3067,16 +3061,16 @@
       <c r="F44" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G44" s="17" t="s">
+      <c r="G44" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17" t="s">
+      <c r="H44" s="28"/>
+      <c r="I44" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
+      <c r="J44" s="28"/>
+      <c r="K44" s="28"/>
+      <c r="L44" s="28"/>
       <c r="M44" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M43,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M43,"-", -1))+1,"0"))</f>
         <v>ex-2</v>
@@ -3084,13 +3078,13 @@
       <c r="N44" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="O44" s="18"/>
+      <c r="O44" s="29"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B45" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C45" s="17" t="s">
+      <c r="C45" s="28" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="3" t="str">
@@ -3103,16 +3097,16 @@
       <c r="F45" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G45" s="17" t="s">
+      <c r="G45" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17" t="s">
+      <c r="H45" s="28"/>
+      <c r="I45" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
+      <c r="J45" s="28"/>
+      <c r="K45" s="28"/>
+      <c r="L45" s="28"/>
       <c r="M45" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M44,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M44,"-", -1))+1,"0"))</f>
         <v>ex-3</v>
@@ -3120,13 +3114,13 @@
       <c r="N45" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="O45" s="18"/>
+      <c r="O45" s="29"/>
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C46" s="17"/>
+      <c r="C46" s="28"/>
       <c r="D46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(D45,LEN(D45)-FIND("~",D45,1))) + 8))</f>
         <v>68~6F</v>
@@ -3137,16 +3131,16 @@
       <c r="F46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G46" s="17" t="s">
+      <c r="G46" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17" t="s">
+      <c r="H46" s="28"/>
+      <c r="I46" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
+      <c r="J46" s="28"/>
+      <c r="K46" s="28"/>
+      <c r="L46" s="28"/>
       <c r="M46" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M45,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M45,"-", -1))+1,"0"))</f>
         <v>ex-4</v>
@@ -3154,13 +3148,13 @@
       <c r="N46" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="O46" s="18"/>
+      <c r="O46" s="29"/>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B47" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C47" s="17"/>
+      <c r="C47" s="28"/>
       <c r="D47" s="4" t="str">
         <f>DEC2HEX(HEX2DEC(RIGHT(D46,LEN(D46)-FIND("~",D46,1))) + 1)</f>
         <v>70</v>
@@ -3171,16 +3165,16 @@
       <c r="F47" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G47" s="17" t="s">
+      <c r="G47" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="H47" s="17"/>
-      <c r="I47" s="17" t="s">
+      <c r="H47" s="28"/>
+      <c r="I47" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
+      <c r="J47" s="28"/>
+      <c r="K47" s="28"/>
+      <c r="L47" s="28"/>
       <c r="M47" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M46,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M46,"-", -1))+1,"0"))</f>
         <v>ex-5</v>
@@ -3188,13 +3182,13 @@
       <c r="N47" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="O47" s="18"/>
+      <c r="O47" s="29"/>
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C48" s="17"/>
+      <c r="C48" s="28"/>
       <c r="D48" s="3" t="str">
         <f t="shared" ref="D48:D54" si="5">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D47)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D47)+1))</f>
         <v>71</v>
@@ -3202,28 +3196,28 @@
       <c r="E48" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="17" t="s">
+      <c r="F48" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G48" s="17"/>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17" t="s">
+      <c r="G48" s="28"/>
+      <c r="H48" s="28"/>
+      <c r="I48" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="17" t="s">
+      <c r="J48" s="28"/>
+      <c r="K48" s="28"/>
+      <c r="L48" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="M48" s="17"/>
-      <c r="N48" s="17"/>
-      <c r="O48" s="18"/>
+      <c r="M48" s="28"/>
+      <c r="N48" s="28"/>
+      <c r="O48" s="29"/>
     </row>
     <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C49" s="17"/>
+      <c r="C49" s="28"/>
       <c r="D49" s="3" t="str">
         <f t="shared" si="5"/>
         <v>72</v>
@@ -3231,32 +3225,32 @@
       <c r="E49" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F49" s="17" t="s">
+      <c r="F49" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17" t="s">
+      <c r="G49" s="28"/>
+      <c r="H49" s="28"/>
+      <c r="I49" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
+      <c r="J49" s="28"/>
+      <c r="K49" s="28"/>
       <c r="L49" s="6" t="s">
         <v>46</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="N49" s="17" t="s">
+      <c r="N49" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="O49" s="18"/>
+      <c r="O49" s="29"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C50" s="17"/>
+      <c r="C50" s="28"/>
       <c r="D50" s="3" t="str">
         <f t="shared" si="5"/>
         <v>73</v>
@@ -3264,32 +3258,32 @@
       <c r="E50" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F50" s="17" t="s">
+      <c r="F50" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17" t="s">
+      <c r="G50" s="28"/>
+      <c r="H50" s="28"/>
+      <c r="I50" s="28" t="s">
         <v>179</v>
       </c>
-      <c r="J50" s="17"/>
-      <c r="K50" s="17"/>
+      <c r="J50" s="28"/>
+      <c r="K50" s="28"/>
       <c r="L50" s="5" t="s">
         <v>107</v>
       </c>
       <c r="M50" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="N50" s="17" t="s">
+      <c r="N50" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="O50" s="18"/>
+      <c r="O50" s="29"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C51" s="17"/>
+      <c r="C51" s="28"/>
       <c r="D51" s="3" t="str">
         <f t="shared" si="5"/>
         <v>74</v>
@@ -3297,16 +3291,16 @@
       <c r="E51" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="F51" s="17" t="s">
+      <c r="F51" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G51" s="17"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="17" t="s">
+      <c r="G51" s="28"/>
+      <c r="H51" s="28"/>
+      <c r="I51" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
+      <c r="J51" s="28"/>
+      <c r="K51" s="28"/>
       <c r="L51" s="5" t="s">
         <v>107</v>
       </c>
@@ -3314,16 +3308,16 @@
         <f t="shared" ref="M51:M59" si="6">_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(M50)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(M50)+1))</f>
         <v>01</v>
       </c>
-      <c r="N51" s="17" t="s">
+      <c r="N51" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="O51" s="18"/>
+      <c r="O51" s="29"/>
     </row>
     <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C52" s="17"/>
+      <c r="C52" s="28"/>
       <c r="D52" s="3" t="str">
         <f t="shared" si="5"/>
         <v>75</v>
@@ -3331,16 +3325,16 @@
       <c r="E52" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F52" s="17" t="s">
+      <c r="F52" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17" t="s">
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
+      <c r="I52" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
+      <c r="J52" s="28"/>
+      <c r="K52" s="28"/>
       <c r="L52" s="5" t="s">
         <v>107</v>
       </c>
@@ -3348,16 +3342,16 @@
         <f t="shared" si="6"/>
         <v>02</v>
       </c>
-      <c r="N52" s="17" t="s">
+      <c r="N52" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="O52" s="18"/>
+      <c r="O52" s="29"/>
     </row>
     <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C53" s="17" t="s">
+      <c r="C53" s="28" t="s">
         <v>50</v>
       </c>
       <c r="D53" s="3" t="str">
@@ -3367,16 +3361,16 @@
       <c r="E53" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F53" s="17" t="s">
+      <c r="F53" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="17" t="s">
+      <c r="G53" s="28"/>
+      <c r="H53" s="28"/>
+      <c r="I53" s="28" t="s">
         <v>180</v>
       </c>
-      <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
+      <c r="J53" s="28"/>
+      <c r="K53" s="28"/>
       <c r="L53" s="5" t="s">
         <v>109</v>
       </c>
@@ -3384,16 +3378,16 @@
         <f t="shared" si="6"/>
         <v>03</v>
       </c>
-      <c r="N53" s="17" t="s">
+      <c r="N53" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="O53" s="18"/>
+      <c r="O53" s="29"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="17"/>
+      <c r="C54" s="28"/>
       <c r="D54" s="3" t="str">
         <f t="shared" si="5"/>
         <v>77</v>
@@ -3401,16 +3395,16 @@
       <c r="E54" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F54" s="17" t="s">
+      <c r="F54" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17" t="s">
+      <c r="G54" s="28"/>
+      <c r="H54" s="28"/>
+      <c r="I54" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="J54" s="17"/>
-      <c r="K54" s="17"/>
+      <c r="J54" s="28"/>
+      <c r="K54" s="28"/>
       <c r="L54" s="5" t="s">
         <v>107</v>
       </c>
@@ -3418,16 +3412,16 @@
         <f t="shared" si="6"/>
         <v>04</v>
       </c>
-      <c r="N54" s="17" t="s">
+      <c r="N54" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="O54" s="18"/>
+      <c r="O54" s="29"/>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C55" s="17"/>
+      <c r="C55" s="28"/>
       <c r="D55" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D54)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D54)+1))</f>
         <v>78</v>
@@ -3444,11 +3438,11 @@
       <c r="H55" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="I55" s="17" t="s">
+      <c r="I55" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="J55" s="17"/>
-      <c r="K55" s="17"/>
+      <c r="J55" s="28"/>
+      <c r="K55" s="28"/>
       <c r="L55" s="5" t="s">
         <v>107</v>
       </c>
@@ -3456,16 +3450,16 @@
         <f t="shared" si="6"/>
         <v>05</v>
       </c>
-      <c r="N55" s="17" t="s">
+      <c r="N55" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="O55" s="18"/>
+      <c r="O55" s="29"/>
     </row>
     <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C56" s="17"/>
+      <c r="C56" s="28"/>
       <c r="D56" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D55)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D55)+1))</f>
         <v>79</v>
@@ -3482,11 +3476,11 @@
       <c r="H56" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="I56" s="17" t="s">
+      <c r="I56" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="J56" s="17"/>
-      <c r="K56" s="17"/>
+      <c r="J56" s="28"/>
+      <c r="K56" s="28"/>
       <c r="L56" s="5" t="s">
         <v>110</v>
       </c>
@@ -3494,16 +3488,16 @@
         <f t="shared" si="6"/>
         <v>06</v>
       </c>
-      <c r="N56" s="17" t="s">
+      <c r="N56" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="O56" s="18"/>
+      <c r="O56" s="29"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="28" t="s">
         <v>47</v>
       </c>
       <c r="D57" s="3" t="str">
@@ -3522,11 +3516,11 @@
       <c r="H57" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="I57" s="17" t="s">
+      <c r="I57" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
+      <c r="J57" s="28"/>
+      <c r="K57" s="28"/>
       <c r="L57" s="5" t="s">
         <v>109</v>
       </c>
@@ -3534,16 +3528,16 @@
         <f t="shared" si="6"/>
         <v>07</v>
       </c>
-      <c r="N57" s="17" t="s">
+      <c r="N57" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="O57" s="18"/>
+      <c r="O57" s="29"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C58" s="17"/>
+      <c r="C58" s="28"/>
       <c r="D58" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,TRUE,IF(HEX2DEC(D57)+1 &lt; 16,"0", ""), DEC2HEX(HEX2DEC(D57)+1))</f>
         <v>7B</v>
@@ -3560,11 +3554,11 @@
       <c r="H58" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="I58" s="17" t="s">
+      <c r="I58" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="J58" s="17"/>
-      <c r="K58" s="17"/>
+      <c r="J58" s="28"/>
+      <c r="K58" s="28"/>
       <c r="L58" s="5" t="s">
         <v>107</v>
       </c>
@@ -3572,16 +3566,16 @@
         <f t="shared" si="6"/>
         <v>08</v>
       </c>
-      <c r="N58" s="17" t="s">
+      <c r="N58" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="O58" s="18"/>
+      <c r="O58" s="29"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C59" s="17" t="s">
+      <c r="C59" s="28" t="s">
         <v>38</v>
       </c>
       <c r="D59" s="3" t="str">
@@ -3591,18 +3585,18 @@
       <c r="E59" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="F59" s="17" t="s">
+      <c r="F59" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G59" s="17"/>
+      <c r="G59" s="28"/>
       <c r="H59" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="I59" s="17" t="s">
+      <c r="I59" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
+      <c r="J59" s="28"/>
+      <c r="K59" s="28"/>
       <c r="L59" s="5" t="s">
         <v>107</v>
       </c>
@@ -3610,16 +3604,16 @@
         <f t="shared" si="6"/>
         <v>09</v>
       </c>
-      <c r="N59" s="17" t="s">
+      <c r="N59" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="O59" s="18"/>
+      <c r="O59" s="29"/>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C60" s="17"/>
+      <c r="C60" s="28"/>
       <c r="D60" s="3" t="str">
         <f t="shared" si="7"/>
         <v>7D</v>
@@ -3636,11 +3630,11 @@
       <c r="H60" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="I60" s="17" t="s">
+      <c r="I60" s="28" t="s">
         <v>185</v>
       </c>
-      <c r="J60" s="17"/>
-      <c r="K60" s="17"/>
+      <c r="J60" s="28"/>
+      <c r="K60" s="28"/>
       <c r="L60" s="5" t="s">
         <v>109</v>
       </c>
@@ -3648,10 +3642,10 @@
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(M59) + 1),"~",DEC2HEX(HEX2DEC(M59) + 6))</f>
         <v>A~F</v>
       </c>
-      <c r="N60" s="17" t="s">
+      <c r="N60" s="28" t="s">
         <v>173</v>
       </c>
-      <c r="O60" s="18"/>
+      <c r="O60" s="29"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B61" s="9" t="s">
@@ -3676,11 +3670,11 @@
       <c r="H61" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="I61" s="17" t="s">
+      <c r="I61" s="28" t="s">
         <v>204</v>
       </c>
-      <c r="J61" s="17"/>
-      <c r="K61" s="17"/>
+      <c r="J61" s="28"/>
+      <c r="K61" s="28"/>
       <c r="L61" s="5" t="s">
         <v>109</v>
       </c>
@@ -3688,10 +3682,10 @@
         <f>_xlfn.TEXTJOIN(,FALSE,DEC2HEX(HEX2DEC(RIGHT(M60,LEN(M60)-FIND("~",M60,1))) + 1),"~",DEC2HEX(HEX2DEC(RIGHT(M60,LEN(M60)-FIND("~",M60,1))) + 16))</f>
         <v>10~1F</v>
       </c>
-      <c r="N61" s="17" t="s">
+      <c r="N61" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="O61" s="18"/>
+      <c r="O61" s="29"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="9" t="s">
@@ -3707,24 +3701,24 @@
       <c r="E62" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="F62" s="17" t="s">
+      <c r="F62" s="28" t="s">
         <v>207</v>
       </c>
-      <c r="G62" s="17"/>
+      <c r="G62" s="28"/>
       <c r="H62" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="I62" s="17" t="s">
+      <c r="I62" s="28" t="s">
         <v>208</v>
       </c>
-      <c r="J62" s="17"/>
-      <c r="K62" s="17"/>
-      <c r="L62" s="17" t="s">
+      <c r="J62" s="28"/>
+      <c r="K62" s="28"/>
+      <c r="L62" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="M62" s="17"/>
-      <c r="N62" s="17"/>
-      <c r="O62" s="18"/>
+      <c r="M62" s="28"/>
+      <c r="N62" s="28"/>
+      <c r="O62" s="29"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="9" t="s">
@@ -3740,16 +3734,16 @@
       <c r="E63" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F63" s="17" t="s">
+      <c r="F63" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="G63" s="17"/>
-      <c r="H63" s="17"/>
-      <c r="I63" s="17" t="s">
+      <c r="G63" s="28"/>
+      <c r="H63" s="28"/>
+      <c r="I63" s="28" t="s">
         <v>192</v>
       </c>
-      <c r="J63" s="17"/>
-      <c r="K63" s="17"/>
+      <c r="J63" s="28"/>
+      <c r="K63" s="28"/>
       <c r="L63" s="5" t="s">
         <v>39</v>
       </c>
@@ -3764,25 +3758,25 @@
       </c>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B64" s="37" t="s">
+      <c r="B64" s="16" t="s">
         <v>209</v>
       </c>
       <c r="C64" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(M47,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(M47,"-", -1))+1,"0"))</f>
         <v>ex-6</v>
       </c>
-      <c r="D64" s="32"/>
-      <c r="E64" s="38" t="s">
+      <c r="D64" s="3"/>
+      <c r="E64" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="F64" s="41"/>
-      <c r="G64" s="29"/>
-      <c r="H64" s="17" t="s">
+      <c r="F64" s="22"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="28" t="s">
         <v>193</v>
       </c>
-      <c r="I64" s="17"/>
-      <c r="J64" s="17"/>
-      <c r="K64" s="17"/>
+      <c r="I64" s="28"/>
+      <c r="J64" s="28"/>
+      <c r="K64" s="28"/>
       <c r="L64" s="4" t="s">
         <v>96</v>
       </c>
@@ -3798,15 +3792,15 @@
       </c>
     </row>
     <row r="65" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B65" s="35"/>
+      <c r="B65" s="17"/>
       <c r="C65" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(C64,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(C64,"-", -1))+1,"0"))</f>
         <v>ex-7</v>
       </c>
-      <c r="D65" s="32"/>
-      <c r="E65" s="39"/>
-      <c r="F65" s="42"/>
-      <c r="G65" s="30"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="24"/>
+      <c r="G65" s="25"/>
       <c r="H65" s="4" t="s">
         <v>203</v>
       </c>
@@ -3835,15 +3829,15 @@
       </c>
     </row>
     <row r="66" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B66" s="35"/>
+      <c r="B66" s="17"/>
       <c r="C66" s="3" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(C65,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(C65,"-", -1))+1,"0"))</f>
         <v>ex-8</v>
       </c>
-      <c r="D66" s="32"/>
-      <c r="E66" s="39"/>
-      <c r="F66" s="42"/>
-      <c r="G66" s="30"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="24"/>
+      <c r="G66" s="25"/>
       <c r="H66" s="3" t="s">
         <v>199</v>
       </c>
@@ -3872,21 +3866,21 @@
       </c>
     </row>
     <row r="67" spans="2:15" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B67" s="36"/>
-      <c r="C67" s="34" t="str">
+      <c r="B67" s="18"/>
+      <c r="C67" s="12" t="str">
         <f>_xlfn.TEXTJOIN(,FALSE,_xlfn.TEXTBEFORE(C66,"-",-1),"-",TEXT(VALUE(_xlfn.TEXTAFTER(C66,"-", -1))+1,"0"))</f>
         <v>ex-9</v>
       </c>
-      <c r="D67" s="34"/>
-      <c r="E67" s="40"/>
-      <c r="F67" s="43"/>
-      <c r="G67" s="31"/>
-      <c r="H67" s="33" t="s">
+      <c r="D67" s="12"/>
+      <c r="E67" s="21"/>
+      <c r="F67" s="26"/>
+      <c r="G67" s="27"/>
+      <c r="H67" s="30" t="s">
         <v>201</v>
       </c>
-      <c r="I67" s="33"/>
-      <c r="J67" s="33"/>
-      <c r="K67" s="33"/>
+      <c r="I67" s="30"/>
+      <c r="J67" s="30"/>
+      <c r="K67" s="30"/>
       <c r="L67" s="12" t="str">
         <f>_xlfn.VALUETOTEXT(L66+1)</f>
         <v>3</v>
@@ -3904,6 +3898,115 @@
     </row>
   </sheetData>
   <mergeCells count="133">
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="L48:O48"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="N56:O56"/>
+    <mergeCell ref="N57:O57"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="U15:AB15"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="T35:V35"/>
+    <mergeCell ref="W35:Y35"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="C45:C52"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="B6:O8"/>
+    <mergeCell ref="I25:K25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I24:K24"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="O16:O23"/>
+    <mergeCell ref="O24:O31"/>
+    <mergeCell ref="L11:L36"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="C11:C36"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="H64:K64"/>
+    <mergeCell ref="H67:K67"/>
+    <mergeCell ref="O12:O15"/>
+    <mergeCell ref="O32:O35"/>
+    <mergeCell ref="O37:O39"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N53:O53"/>
     <mergeCell ref="B64:B67"/>
     <mergeCell ref="E64:E67"/>
     <mergeCell ref="F64:G67"/>
@@ -3928,115 +4031,6 @@
     <mergeCell ref="I54:K54"/>
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="C53:C56"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="H64:K64"/>
-    <mergeCell ref="H67:K67"/>
-    <mergeCell ref="O12:O15"/>
-    <mergeCell ref="O32:O35"/>
-    <mergeCell ref="O37:O39"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N54:O54"/>
-    <mergeCell ref="B6:O8"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="O16:O23"/>
-    <mergeCell ref="O24:O31"/>
-    <mergeCell ref="L11:L36"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="C11:C36"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="U15:AB15"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="T35:V35"/>
-    <mergeCell ref="W35:Y35"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="C45:C52"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="AF15:AG15"/>
-    <mergeCell ref="L48:O48"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="N56:O56"/>
-    <mergeCell ref="N57:O57"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="T34:V34"/>
-    <mergeCell ref="W34:Y34"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="I52:K52"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>